<commit_message>
Normalize line endings and add home/cart/contact UI fixes
Includes pre-existing line-ending normalization across the tree plus
this session's fixes: home page stats bar and JSON-LD, corrected
Vision section image, cart empty-state content, and a Google Maps
embed on the contact page.
</commit_message>
<xml_diff>
--- a/PRICE LISTS.xlsx
+++ b/PRICE LISTS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\navin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\best pneumatics\best-pneumatics-store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759B38BC-75B7-43AE-886C-CD677988A57B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C03DD55-3962-4DB5-9D5B-CE35CD4856FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="937" xr2:uid="{4A3E726E-8BDA-491F-9C01-2728E0B892C3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="937" firstSheet="6" activeTab="16" xr2:uid="{4A3E726E-8BDA-491F-9C01-2728E0B892C3}"/>
   </bookViews>
   <sheets>
     <sheet name="PU-SEAL" sheetId="18" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="296">
   <si>
     <t>2.1-3.5MM</t>
   </si>
@@ -943,6 +943,9 @@
   </si>
   <si>
     <t>SIZE DESCRIPTION (inner x outer dia)</t>
+  </si>
+  <si>
+    <t>stainless steel</t>
   </si>
 </sst>
 </file>
@@ -1509,15 +1512,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1574,6 +1568,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2005,43 +2008,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="30.75" customHeight="1" x14ac:dyDescent="0.8">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="45" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
       <c r="V1"/>
       <c r="AB1"/>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="46" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="49" t="s">
+      <c r="C2" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="D2" s="49" t="s">
+      <c r="D2" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49" t="s">
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46" t="s">
         <v>57</v>
       </c>
       <c r="V2"/>
       <c r="AB2"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A3" s="49"/>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
+      <c r="A3" s="46"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
       <c r="D3" s="34" t="s">
         <v>158</v>
       </c>
@@ -2051,7 +2054,7 @@
       <c r="F3" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="G3" s="49"/>
+      <c r="G3" s="46"/>
       <c r="V3"/>
       <c r="AB3"/>
     </row>
@@ -10039,12 +10042,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
     </row>
     <row r="2" spans="1:4" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
@@ -10139,11 +10142,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
     </row>
     <row r="2" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
@@ -10250,10 +10253,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="45.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="52" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="55"/>
+      <c r="B1" s="52"/>
     </row>
     <row r="2" spans="1:2" ht="36.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
@@ -10348,11 +10351,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
@@ -10543,12 +10546,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
@@ -10974,11 +10977,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="55" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="56"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
@@ -11097,12 +11100,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="57" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
     </row>
     <row r="2" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
@@ -11259,12 +11262,12 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="58" t="s">
         <v>153</v>
       </c>
-      <c r="B14" s="61"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
+      <c r="B14" s="58"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
@@ -11369,10 +11372,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="31.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="52" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="55"/>
+      <c r="B1" s="52"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
@@ -11568,12 +11571,12 @@
   <sheetData>
     <row r="9" spans="1:6" ht="2.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="62" t="s">
+      <c r="A10" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
       <c r="F10" s="20"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -11591,12 +11594,12 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="60" t="s">
         <v>171</v>
       </c>
-      <c r="B12" s="64"/>
-      <c r="C12" s="64"/>
-      <c r="D12" s="65"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="62"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="17">
@@ -11654,15 +11657,18 @@
         <v>640</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="63" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="60" t="s">
         <v>170</v>
       </c>
-      <c r="B17" s="64"/>
-      <c r="C17" s="64"/>
-      <c r="D17" s="65"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="62"/>
+      <c r="E17" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="17">
         <v>1</v>
       </c>
@@ -11676,7 +11682,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="17">
         <v>2</v>
       </c>
@@ -11690,7 +11696,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="17">
         <v>3</v>
       </c>
@@ -11704,7 +11710,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="17">
         <v>4</v>
       </c>
@@ -11718,15 +11724,15 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="64" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="61" t="s">
         <v>173</v>
       </c>
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="61"/>
+      <c r="C22" s="61"/>
+      <c r="D22" s="61"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="17">
         <v>1</v>
       </c>
@@ -11740,7 +11746,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="17">
         <v>2</v>
       </c>
@@ -11754,7 +11760,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="17">
         <v>3</v>
       </c>
@@ -11768,7 +11774,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="17">
         <v>4</v>
       </c>
@@ -11782,7 +11788,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="D30" s="44">
         <v>0.05</v>
       </c>
@@ -11810,14 +11816,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="63" t="s">
         <v>210</v>
       </c>
-      <c r="B2" s="66"/>
+      <c r="B2" s="63"/>
     </row>
     <row r="3" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="66"/>
-      <c r="B3" s="66"/>
+      <c r="A3" s="63"/>
+      <c r="B3" s="63"/>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="18" t="s">
@@ -12414,15 +12420,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="42" customHeight="1" x14ac:dyDescent="1">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="64" t="s">
         <v>212</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="47"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="30" t="s">
@@ -13188,11 +13194,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
@@ -13538,11 +13544,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
     </row>
     <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
@@ -13600,11 +13606,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
     </row>
     <row r="10" spans="1:3" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
@@ -13671,12 +13677,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="51" t="s">
         <v>285</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
@@ -13932,32 +13938,32 @@
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="49" t="s">
         <v>265</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="52"/>
-      <c r="B25" s="52"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
+      <c r="A25" s="49"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="53" t="s">
+      <c r="A26" s="50" t="s">
         <v>266</v>
       </c>
-      <c r="B26" s="53"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="53"/>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
+      <c r="A27" s="50"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -14132,11 +14138,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
     </row>
     <row r="2" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">

</xml_diff>